<commit_message>
Dashboard update 2026-03-16 22:03:05.61
</commit_message>
<xml_diff>
--- a/Movies and Music.xlsx
+++ b/Movies and Music.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kroon\.gemini\antigravity\playground\Books Movies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77BF8770-56EB-4769-B0B9-9543B1F60BAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BFA758C-C043-405E-8552-6DF3D5F68BBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Movies" sheetId="1" r:id="rId1"/>
     <sheet name="TV" sheetId="5" r:id="rId2"/>
     <sheet name="Books" sheetId="2" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="6" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Movies!$A$1:$F$432</definedName>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1114" uniqueCount="554">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1120" uniqueCount="559">
   <si>
     <t>Rating</t>
   </si>
@@ -1704,6 +1705,21 @@
   </si>
   <si>
     <t>Director</t>
+  </si>
+  <si>
+    <t>Loose Change</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Topic</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>PG</t>
   </si>
 </sst>
 </file>
@@ -8897,7 +8913,7 @@
   <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="1" max="1" width="27.28515625" customWidth="1"/>
     <col min="2" max="2" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32.140625" bestFit="1" customWidth="1"/>
   </cols>
@@ -8916,4 +8932,48 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8CA9B39-F148-4282-B30F-098DCE817F14}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="27.28515625" customWidth="1"/>
+    <col min="2" max="2" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>555</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>556</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>554</v>
+      </c>
+      <c r="B2">
+        <v>911</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>558</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Dashboard update 2026-03-17 18:28:37.93
</commit_message>
<xml_diff>
--- a/Movies and Music.xlsx
+++ b/Movies and Music.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kroon\.gemini\antigravity\playground\Books Movies\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BFA758C-C043-405E-8552-6DF3D5F68BBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{756E1F0A-F264-4123-BAE6-E5718EE90EF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Movies" sheetId="1" r:id="rId1"/>
     <sheet name="TV" sheetId="5" r:id="rId2"/>
     <sheet name="Books" sheetId="2" r:id="rId3"/>
-    <sheet name="Sheet1" sheetId="6" r:id="rId4"/>
+    <sheet name="Misc" sheetId="6" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Movies!$A$1:$F$432</definedName>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1120" uniqueCount="559">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1121" uniqueCount="560">
   <si>
     <t>Rating</t>
   </si>
@@ -1719,7 +1719,10 @@
     <t>Link</t>
   </si>
   <si>
-    <t>PG</t>
+    <t>Everything is a Rich Man's Trick</t>
+  </si>
+  <si>
+    <t>Tin Foil</t>
   </si>
 </sst>
 </file>
@@ -8936,10 +8939,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8CA9B39-F148-4282-B30F-098DCE817F14}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.28515625" customWidth="1"/>
+    <col min="1" max="1" width="30.85546875" customWidth="1"/>
     <col min="2" max="2" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="38.7109375" customWidth="1"/>
   </cols>
@@ -8959,18 +8962,16 @@
       <c r="A2" t="s">
         <v>554</v>
       </c>
-      <c r="B2">
-        <v>911</v>
+      <c r="B2" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>558</v>
+      </c>
       <c r="B3" t="s">
-        <v>558</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
     </row>
   </sheetData>

</xml_diff>